<commit_message>
Finished revis NG Inprocess
</commit_message>
<xml_diff>
--- a/bin/Debug/Template/ReportNGTemplate.xlsx
+++ b/bin/Debug/Template/ReportNGTemplate.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project\MC-Dept-App\bin\Debug\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE3F6FB7-22C9-426B-A9B7-F1404432D138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47CDC7BA-E834-46A8-A988-5CA11AE4D66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{5CB8BC32-B174-403D-997B-E960FC6DE88B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5CB8BC32-B174-403D-997B-E960FC6DE88B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sub Part" sheetId="3" r:id="rId1"/>
     <sheet name="RM" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">RM!$A$1:$H$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">RM!$A$1:$I$48</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Sub Part'!$A$1:$G$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="16">
   <si>
     <t>POSC</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t>27-07-2026 ~ 28-08-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RM Name </t>
   </si>
 </sst>
 </file>
@@ -319,22 +322,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>655865</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>99391</xdr:rowOff>
+      <xdr:rowOff>99392</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>629316</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>538207</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>99392</xdr:rowOff>
+      <xdr:rowOff>99393</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="2" name="Group 1">
+        <xdr:cNvPr id="3" name="Group 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93E6F039-99B9-3F45-81B2-8BD87B913254}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52B8A6D2-5FD9-EF01-3601-C84043B17AE9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -342,245 +345,12 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="0" y="670891"/>
-          <a:ext cx="6592794" cy="952501"/>
-          <a:chOff x="0" y="670891"/>
-          <a:chExt cx="6592794" cy="952501"/>
+          <a:off x="655865" y="670892"/>
+          <a:ext cx="6119146" cy="952501"/>
+          <a:chOff x="1384735" y="670891"/>
+          <a:chExt cx="5208059" cy="952501"/>
         </a:xfrm>
       </xdr:grpSpPr>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="91" name="Rectangle 90">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F583495A-4E7B-5E2E-3266-B830A4D07792}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="41123" y="681632"/>
-            <a:ext cx="1231985" cy="906517"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:gradFill flip="none" rotWithShape="1">
-            <a:gsLst>
-              <a:gs pos="0">
-                <a:srgbClr val="FF0000">
-                  <a:shade val="30000"/>
-                  <a:satMod val="115000"/>
-                </a:srgbClr>
-              </a:gs>
-              <a:gs pos="50000">
-                <a:srgbClr val="FF0000">
-                  <a:shade val="67500"/>
-                  <a:satMod val="115000"/>
-                </a:srgbClr>
-              </a:gs>
-              <a:gs pos="100000">
-                <a:srgbClr val="FF0000">
-                  <a:shade val="100000"/>
-                  <a:satMod val="115000"/>
-                </a:srgbClr>
-              </a:gs>
-            </a:gsLst>
-            <a:lin ang="2700000" scaled="1"/>
-            <a:tileRect/>
-          </a:gradFill>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="2">
-            <a:schemeClr val="accent1">
-              <a:shade val="15000"/>
-            </a:schemeClr>
-          </a:lnRef>
-          <a:fillRef idx="1">
-            <a:schemeClr val="accent1"/>
-          </a:fillRef>
-          <a:effectRef idx="0">
-            <a:schemeClr val="accent1"/>
-          </a:effectRef>
-          <a:fontRef idx="minor">
-            <a:schemeClr val="lt1"/>
-          </a:fontRef>
-        </xdr:style>
-        <xdr:txBody>
-          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:endParaRPr lang="en-US" sz="1100"/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="92" name="Rectangle 91">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D1D521D7-6186-C621-7393-B6049CAC8817}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="32840" y="710640"/>
-            <a:ext cx="1228183" cy="230832"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr"/>
-            <a:r>
-              <a:rPr lang="en-US" sz="900" b="0" u="sng" cap="none" spc="0">
-                <a:ln w="0">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>STOP</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" sz="900" b="0" u="sng" cap="none" spc="0" baseline="0">
-                <a:ln w="0">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t> INFORMATION</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US" sz="900" b="0" u="sng" cap="none" spc="0">
-              <a:ln w="0">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="$I$7">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="93" name="plan">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BB035CF-04B6-A05D-D970-8A2667057CC5}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="651985" y="1061996"/>
-            <a:ext cx="644657" cy="205697"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:fld id="{4616CBF4-C6AD-41AA-983E-C834EB97F8B3}" type="TxLink">
-              <a:rPr lang="en-US" sz="700" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Calibri"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:rPr>
-              <a:pPr algn="l"/>
-              <a:t>Plan</a:t>
-            </a:fld>
-            <a:endParaRPr lang="en-US" sz="100" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
       <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
           <xdr:cNvPr id="94" name="Rectangle 93">
@@ -1441,511 +1211,6 @@
           </a:p>
         </xdr:txBody>
       </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="106" name="Rectangle 105">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54EEAA09-2771-E808-97B7-EB34685BB417}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="0" y="1357002"/>
-            <a:ext cx="791727" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>Machine</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t> Broken :</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="107" name="Rectangle 106">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4BBE211-208C-B303-4396-77962841E63D}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="0" y="1212966"/>
-            <a:ext cx="784114" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>Production</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t> NG    :</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="108" name="Rectangle 107">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B8FF6533-CD89-8523-B280-2B60AADD2645}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="0" y="1059636"/>
-            <a:ext cx="799339" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>Change Plan       :</a:t>
-            </a:r>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="109" name="Rectangle 108">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{88BC4A84-0E4D-8142-F466-FCC402ECFF46}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="0" y="910953"/>
-            <a:ext cx="795533" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>Change Wire       :</a:t>
-            </a:r>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="$I$6">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="110" name="wire">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D35DB98-F1DA-D411-CC5D-F13572AC0FDF}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="658798" y="908130"/>
-            <a:ext cx="644156" cy="205697"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:fld id="{38772519-C104-45CF-A119-505635CC44CC}" type="TxLink">
-              <a:rPr lang="en-US" sz="700" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Calibri"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:rPr>
-              <a:pPr algn="l"/>
-              <a:t>Wire</a:t>
-            </a:fld>
-            <a:endParaRPr lang="en-US" sz="100" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="#REF!">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="111" name="ng">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{614C8FA3-52D7-CC84-791D-57DD5FA8B660}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="644158" y="1215861"/>
-            <a:ext cx="644156" cy="205697"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:fld id="{6887CB99-FA84-41FA-8064-312979EDAD6E}" type="TxLink">
-              <a:rPr lang="en-US" sz="700" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Calibri"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:rPr>
-              <a:pPr algn="l"/>
-              <a:t>NG</a:t>
-            </a:fld>
-            <a:endParaRPr lang="en-US" sz="100" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="$I$9">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="112" name="broken">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{38A71FAD-F720-3033-6742-6CCCDC50E240}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="644158" y="1362399"/>
-            <a:ext cx="644156" cy="205697"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:fld id="{0C13CF06-D83C-4A4F-AF60-7C1D3AC11532}" type="TxLink">
-              <a:rPr lang="en-US" sz="700" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Calibri"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:rPr>
-              <a:pPr algn="l"/>
-              <a:t>MC</a:t>
-            </a:fld>
-            <a:endParaRPr lang="en-US" sz="100" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift Light SemiCondensed" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
     </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
@@ -1957,22 +1222,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>751815</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>112360</xdr:rowOff>
+      <xdr:rowOff>104078</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3828</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>525632</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>92884</xdr:rowOff>
+      <xdr:rowOff>84602</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="3" name="Group 2">
+        <xdr:cNvPr id="4" name="Group 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FAC258DD-A45F-3892-2180-C62F3AC805AE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB767385-B2E2-5A6E-5E57-BC20A7707D9A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1980,245 +1245,12 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="0" y="683860"/>
-          <a:ext cx="6613350" cy="933024"/>
-          <a:chOff x="0" y="683860"/>
-          <a:chExt cx="6613350" cy="933024"/>
+          <a:off x="751815" y="675578"/>
+          <a:ext cx="6921708" cy="933024"/>
+          <a:chOff x="1538663" y="683860"/>
+          <a:chExt cx="5786991" cy="933024"/>
         </a:xfrm>
       </xdr:grpSpPr>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="2" name="Rectangle 1">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45D2CB2A-9EEC-E9E1-6A58-BAADCFA8F643}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="41251" y="695457"/>
-            <a:ext cx="1235827" cy="906517"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:gradFill flip="none" rotWithShape="1">
-            <a:gsLst>
-              <a:gs pos="0">
-                <a:srgbClr val="FF0000">
-                  <a:shade val="30000"/>
-                  <a:satMod val="115000"/>
-                </a:srgbClr>
-              </a:gs>
-              <a:gs pos="50000">
-                <a:srgbClr val="FF0000">
-                  <a:shade val="67500"/>
-                  <a:satMod val="115000"/>
-                </a:srgbClr>
-              </a:gs>
-              <a:gs pos="100000">
-                <a:srgbClr val="FF0000">
-                  <a:shade val="100000"/>
-                  <a:satMod val="115000"/>
-                </a:srgbClr>
-              </a:gs>
-            </a:gsLst>
-            <a:lin ang="2700000" scaled="1"/>
-            <a:tileRect/>
-          </a:gradFill>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="2">
-            <a:schemeClr val="accent1">
-              <a:shade val="15000"/>
-            </a:schemeClr>
-          </a:lnRef>
-          <a:fillRef idx="1">
-            <a:schemeClr val="accent1"/>
-          </a:fillRef>
-          <a:effectRef idx="0">
-            <a:schemeClr val="accent1"/>
-          </a:effectRef>
-          <a:fontRef idx="minor">
-            <a:schemeClr val="lt1"/>
-          </a:fontRef>
-        </xdr:style>
-        <xdr:txBody>
-          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:endParaRPr lang="en-US" sz="1100"/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="14" name="Rectangle 13">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D033B12C-C80A-8597-07C5-6F592A261A93}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="32943" y="724465"/>
-            <a:ext cx="1232012" cy="230832"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr"/>
-            <a:r>
-              <a:rPr lang="en-US" sz="900" b="0" u="sng" cap="none" spc="0">
-                <a:ln w="0">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>STOP</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" sz="900" b="0" u="sng" cap="none" spc="0" baseline="0">
-                <a:ln w="0">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t> INFORMATION</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US" sz="900" b="0" u="sng" cap="none" spc="0">
-              <a:ln w="0">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="$J$7">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="62" name="plan">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A791331F-D490-D733-89A2-B41CD503BB5C}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="654018" y="1078643"/>
-            <a:ext cx="646667" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:fld id="{674C6007-E5B4-4E15-AF2E-87D84C800216}" type="TxLink">
-              <a:rPr lang="en-US" sz="700" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:rPr>
-              <a:pPr algn="l"/>
-              <a:t>Plan</a:t>
-            </a:fld>
-            <a:endParaRPr lang="en-US" sz="200" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
       <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
           <xdr:cNvPr id="9" name="Rectangle 8">
@@ -2232,8 +1264,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="1389079" y="698770"/>
-            <a:ext cx="1237013" cy="906517"/>
+            <a:off x="1538693" y="698770"/>
+            <a:ext cx="1370248" cy="906517"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2301,8 +1333,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="4053930" y="695739"/>
-            <a:ext cx="1236098" cy="921145"/>
+            <a:off x="4490567" y="695739"/>
+            <a:ext cx="1369234" cy="921145"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2370,8 +1402,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="2742212" y="695740"/>
-            <a:ext cx="1238620" cy="919370"/>
+            <a:off x="3037567" y="695740"/>
+            <a:ext cx="1372028" cy="919370"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2445,8 +1477,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="5377206" y="683860"/>
-            <a:ext cx="1236144" cy="906517"/>
+            <a:off x="5956369" y="683860"/>
+            <a:ext cx="1369285" cy="906517"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2514,8 +1546,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="1389052" y="711327"/>
-            <a:ext cx="1231055" cy="230832"/>
+            <a:off x="1538663" y="711327"/>
+            <a:ext cx="1363648" cy="230832"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2605,8 +1637,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="4052355" y="727894"/>
-            <a:ext cx="1231055" cy="230832"/>
+            <a:off x="4488822" y="727894"/>
+            <a:ext cx="1363648" cy="230832"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2696,8 +1728,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="2740011" y="729607"/>
-            <a:ext cx="1231055" cy="230832"/>
+            <a:off x="3035129" y="729607"/>
+            <a:ext cx="1363648" cy="230832"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2748,8 +1780,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="5371877" y="698189"/>
-            <a:ext cx="1231055" cy="230832"/>
+            <a:off x="5950466" y="698189"/>
+            <a:ext cx="1363648" cy="230832"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2787,7 +1819,7 @@
           </a:p>
         </xdr:txBody>
       </xdr:sp>
-      <xdr:sp macro="" textlink="$J$2">
+      <xdr:sp macro="" textlink="$K$2">
         <xdr:nvSpPr>
           <xdr:cNvPr id="19" name="ttlsubqty">
             <a:extLst>
@@ -2800,8 +1832,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="1395635" y="1018760"/>
-            <a:ext cx="1231055" cy="338554"/>
+            <a:off x="1545955" y="1018760"/>
+            <a:ext cx="1363648" cy="338554"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2860,7 +1892,7 @@
           </a:p>
         </xdr:txBody>
       </xdr:sp>
-      <xdr:sp macro="" textlink="$J$3">
+      <xdr:sp macro="" textlink="$K$3">
         <xdr:nvSpPr>
           <xdr:cNvPr id="21" name="ttlrmqty">
             <a:extLst>
@@ -2873,8 +1905,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="4058937" y="1041896"/>
-            <a:ext cx="1231055" cy="338554"/>
+            <a:off x="4496113" y="1041896"/>
+            <a:ext cx="1363648" cy="338554"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2933,7 +1965,7 @@
           </a:p>
         </xdr:txBody>
       </xdr:sp>
-      <xdr:sp macro="" textlink="$J$4">
+      <xdr:sp macro="" textlink="$K$4">
         <xdr:nvSpPr>
           <xdr:cNvPr id="29" name="ttlsubprice">
             <a:extLst>
@@ -2946,8 +1978,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="2733426" y="1043609"/>
-            <a:ext cx="1231055" cy="338554"/>
+            <a:off x="3027835" y="1043609"/>
+            <a:ext cx="1363648" cy="338554"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -3006,7 +2038,7 @@
           </a:p>
         </xdr:txBody>
       </xdr:sp>
-      <xdr:sp macro="" textlink="$J$5">
+      <xdr:sp macro="" textlink="$K$5">
         <xdr:nvSpPr>
           <xdr:cNvPr id="30" name="ttlcostng">
             <a:extLst>
@@ -3019,8 +2051,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="5378459" y="1025328"/>
-            <a:ext cx="1231055" cy="338554"/>
+            <a:off x="5957757" y="1025328"/>
+            <a:ext cx="1363648" cy="338554"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -3079,523 +2111,18 @@
           </a:p>
         </xdr:txBody>
       </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="32" name="Rectangle 31">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5161318-C45E-DBDF-83EA-B78B4B685F47}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="0" y="1370827"/>
-            <a:ext cx="794195" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>Machine</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t> Broken :</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="33" name="Rectangle 32">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A966B2D-C83D-D549-5B6E-2343EC14985A}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="0" y="1226791"/>
-            <a:ext cx="786559" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>Production</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t> NG    :</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="34" name="Rectangle 33">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3670E91D-F3E3-F941-C864-AD136BB2D31F}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="0" y="1073461"/>
-            <a:ext cx="801832" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>Change Plan       :</a:t>
-            </a:r>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="56" name="Rectangle 55">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D93FFBA2-26CE-54AD-AA90-2D2D9457E92E}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="0" y="924778"/>
-            <a:ext cx="798014" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:r>
-              <a:rPr lang="en-US" sz="700" b="0" u="none" cap="none" spc="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight SemiConde" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>Change Wire       :</a:t>
-            </a:r>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="$J$6">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="59" name="wire">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0F45507A-7468-5769-093C-8EE28B13FDB8}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="660852" y="924777"/>
-            <a:ext cx="646165" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:fld id="{439AE9AE-DE40-4300-A508-1B2F50D4DC37}" type="TxLink">
-              <a:rPr lang="en-US" sz="700" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:rPr>
-              <a:pPr algn="l"/>
-              <a:t>Wire</a:t>
-            </a:fld>
-            <a:endParaRPr lang="en-US" sz="200" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="$J$8">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="63" name="ng">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{48F9FF82-FF80-AD2E-DB84-18F0471890C0}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="646167" y="1232508"/>
-            <a:ext cx="646165" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:fld id="{F3ECBCBF-A261-48F1-A850-ECB80257E1E2}" type="TxLink">
-              <a:rPr lang="en-US" sz="700" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift SemiLight" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:rPr>
-              <a:pPr algn="l"/>
-              <a:t>NG</a:t>
-            </a:fld>
-            <a:endParaRPr lang="en-US" sz="200" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift SemiLight" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="$J$9">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="64" name="broken">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB91FB66-1CC4-3C54-CA58-B6300FE5E271}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="646167" y="1379046"/>
-            <a:ext cx="646165" cy="200055"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:fld id="{CF6EAE03-B29A-4ED7-8C7C-FE63FCA0E96D}" type="TxLink">
-              <a:rPr lang="en-US" sz="700" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" baseline="0">
-                <a:ln w="3175">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:ln>
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                    <a:schemeClr val="dk1">
-                      <a:alpha val="40000"/>
-                    </a:schemeClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="Bahnschrift Light SemiCondensed" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
-              </a:rPr>
-              <a:pPr algn="l"/>
-              <a:t>MC</a:t>
-            </a:fld>
-            <a:endParaRPr lang="en-US" sz="200" b="0" u="none" cap="none" spc="0">
-              <a:ln w="3175">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="Bahnschrift Light SemiCondensed" panose="020B0502040204020203" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
     </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>1309687</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>-8238</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1994709" cy="270459"/>
-    <xdr:sp macro="" textlink="$K$2">
+    <xdr:sp macro="" textlink="$L$2">
       <xdr:nvSpPr>
         <xdr:cNvPr id="67" name="Rectangle 66">
           <a:extLst>
@@ -3970,11 +2497,10 @@
   <cols>
     <col min="1" max="1" width="18.7109375" style="10" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="10" customWidth="1"/>
-    <col min="3" max="3" width="16.85546875" style="10" customWidth="1"/>
-    <col min="4" max="4" width="20.85546875" style="10" customWidth="1"/>
+    <col min="3" max="4" width="25.7109375" style="10" customWidth="1"/>
     <col min="5" max="5" width="10.7109375" customWidth="1"/>
     <col min="6" max="6" width="9.5703125" style="8" customWidth="1"/>
-    <col min="7" max="7" width="10" style="10" customWidth="1"/>
+    <col min="7" max="7" width="12.5703125" style="10" customWidth="1"/>
     <col min="8" max="8" width="9.140625" customWidth="1"/>
     <col min="9" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
@@ -4072,7 +2598,7 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="99" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="85" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -4082,22 +2608,21 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" style="10" customWidth="1"/>
-    <col min="2" max="3" width="10.7109375" style="10" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" style="10" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" style="10" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" customWidth="1"/>
-    <col min="8" max="8" width="10" style="10" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="10.7109375" style="10" customWidth="1"/>
+    <col min="5" max="6" width="25.7109375" style="10" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="9.5703125" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" style="10" customWidth="1"/>
+    <col min="10" max="10" width="9.140625" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>7</v>
       </c>
@@ -4108,44 +2633,45 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
       <c r="H1" s="12"/>
-      <c r="I1" s="1"/>
+      <c r="I1" s="12"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="J2" s="4" t="s">
+    <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="7">
+      <c r="L2" s="7">
         <v>46200</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="J3" s="4" t="s">
+    <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="J4" s="4" t="s">
+    <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K4" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="J5" s="4" t="s">
+    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K5" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="J6" s="4" t="s">
+    <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K6" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="J7" s="4" t="s">
+    <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K7" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>0</v>
       </c>
@@ -4156,43 +2682,47 @@
         <v>8</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="K8" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
       <c r="E9" s="11"/>
-      <c r="F9" s="3"/>
+      <c r="F9" s="11"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="11"/>
-      <c r="J9" s="4" t="s">
+      <c r="H9" s="3"/>
+      <c r="I9" s="11"/>
+      <c r="K9" s="4" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="99" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="76" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>